<commit_message>
add new edited version of run analysis
</commit_message>
<xml_diff>
--- a/ML_Projekt run analysis.xlsx
+++ b/ML_Projekt run analysis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Valentin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Valentin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C452DA71-9E79-40B8-8FD0-C1017E87D23F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC544B90-F3AC-4874-9A7E-3E59EC3D317F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{2B83F912-C77A-4961-8D85-54C81C8A018C}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="45">
   <si>
     <t>epochs</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>ResNet50 implemtentation</t>
+  </si>
+  <si>
+    <t>69.96%</t>
   </si>
 </sst>
 </file>
@@ -2004,10 +2007,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2836,7 +2835,7 @@
         <v>19</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>42</v>
@@ -2989,12 +2988,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d117f3be-a310-4f47-998c-7b14ba109482" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3154,17 +3152,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d117f3be-a310-4f47-998c-7b14ba109482" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37B3B558-A0CF-4BE6-90C6-919AD6A7F8AA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FEBA76D8-6634-41BB-AFB1-3345A2853009}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="d117f3be-a310-4f47-998c-7b14ba109482"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3188,17 +3195,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FEBA76D8-6634-41BB-AFB1-3345A2853009}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37B3B558-A0CF-4BE6-90C6-919AD6A7F8AA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="d117f3be-a310-4f47-998c-7b14ba109482"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>